<commit_message>
Swap serisi web arşivinden 2022'ye geri dolduruldu (24 nokta)
- Wayback Machine'deki eski URDL şablonları tarandı; 2022, 2023 ve 2025
  dosyalarından 21 tarihsel dönem kurtarıldı (bozuk capture'lar alternatif
  snapshot'larla, eski metin-tarihli şablon parser düzeltmesiyle çözüldü)
- kolon_tarihi artık '13.05.2022' biçimli metin tarihleri de tanıyor
- EVDS çekimi pencerelere bölündü (API ~1000 satır sınırı): günlük NUR/altın
  serisi artık 2022 başından itibaren — 2022 likidite noktaları eşleşebiliyor
- Seyrek tarihsel seri için ch4/f4 bar yerine çizgi+işaretçi oldu

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/net rezerv/likidite.xlsx
+++ b/net rezerv/likidite.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,70 +471,553 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46203</v>
+        <v>44620</v>
       </c>
       <c r="B2" t="n">
-        <v>147426</v>
+        <v>112335</v>
       </c>
       <c r="C2" t="n">
-        <v>45537</v>
+        <v>60961</v>
       </c>
       <c r="D2" t="n">
-        <v>94250</v>
+        <v>43535</v>
       </c>
       <c r="E2" t="n">
-        <v>-17667</v>
+        <v>-57729</v>
       </c>
       <c r="F2" t="n">
-        <v>1806</v>
+        <v>-3153</v>
       </c>
       <c r="G2" t="n">
-        <v>-15861</v>
+        <v>-60882</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46206</v>
+        <v>44624</v>
       </c>
       <c r="B3" t="n">
-        <v>159694</v>
+        <v>110261</v>
       </c>
       <c r="C3" t="n">
-        <v>54276</v>
+        <v>60319</v>
       </c>
       <c r="D3" t="n">
-        <v>97742</v>
+        <v>42081</v>
       </c>
       <c r="E3" t="n">
-        <v>-17580</v>
+        <v>-57267</v>
       </c>
       <c r="F3" t="n">
-        <v>2535</v>
+        <v>-3528</v>
       </c>
       <c r="G3" t="n">
-        <v>-15045</v>
+        <v>-60795</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
+        <v>44631</v>
+      </c>
+      <c r="B4" t="n">
+        <v>108864</v>
+      </c>
+      <c r="C4" t="n">
+        <v>57497</v>
+      </c>
+      <c r="D4" t="n">
+        <v>43528</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-55770</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-3971</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-59741</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>44638</v>
+      </c>
+      <c r="B5" t="n">
+        <v>108708</v>
+      </c>
+      <c r="C5" t="n">
+        <v>58677</v>
+      </c>
+      <c r="D5" t="n">
+        <v>42208</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-58845</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-3659</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-62504</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>44680</v>
+      </c>
+      <c r="B6" t="n">
+        <v>106858</v>
+      </c>
+      <c r="C6" t="n">
+        <v>57850</v>
+      </c>
+      <c r="D6" t="n">
+        <v>41467</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-61109</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-3502</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-64611</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>44687</v>
+      </c>
+      <c r="B7" t="n">
+        <v>107660</v>
+      </c>
+      <c r="C7" t="n">
+        <v>58413</v>
+      </c>
+      <c r="D7" t="n">
+        <v>41641</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-59806</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-3528</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-63334</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>44694</v>
+      </c>
+      <c r="B8" t="n">
+        <v>101941</v>
+      </c>
+      <c r="C8" t="n">
+        <v>53657</v>
+      </c>
+      <c r="D8" t="n">
+        <v>40743</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-60032</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-3696</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-63728</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>44701</v>
+      </c>
+      <c r="B9" t="n">
+        <v>100261</v>
+      </c>
+      <c r="C9" t="n">
+        <v>52442</v>
+      </c>
+      <c r="D9" t="n">
+        <v>40250</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-60861</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-3829</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-64690</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>44708</v>
+      </c>
+      <c r="B10" t="n">
+        <v>102896</v>
+      </c>
+      <c r="C10" t="n">
+        <v>53656</v>
+      </c>
+      <c r="D10" t="n">
+        <v>41611</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-60788</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-3815</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-64603</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>44985</v>
+      </c>
+      <c r="B11" t="n">
+        <v>117406</v>
+      </c>
+      <c r="C11" t="n">
+        <v>61290</v>
+      </c>
+      <c r="D11" t="n">
+        <v>48661</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-59164</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-3160</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-62324</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>44988</v>
+      </c>
+      <c r="B12" t="n">
+        <v>120359</v>
+      </c>
+      <c r="C12" t="n">
+        <v>62761</v>
+      </c>
+      <c r="D12" t="n">
+        <v>50078</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-61302</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-3187</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-64489</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>45009</v>
+      </c>
+      <c r="B13" t="n">
+        <v>124694</v>
+      </c>
+      <c r="C13" t="n">
+        <v>63711</v>
+      </c>
+      <c r="D13" t="n">
+        <v>53358</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-57225</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-3364</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-60589</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>45838</v>
+      </c>
+      <c r="B14" t="n">
+        <v>149897</v>
+      </c>
+      <c r="C14" t="n">
+        <v>59070</v>
+      </c>
+      <c r="D14" t="n">
+        <v>83093</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-19499</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1663</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-17836</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>45842</v>
+      </c>
+      <c r="B15" t="n">
+        <v>164397</v>
+      </c>
+      <c r="C15" t="n">
+        <v>72002</v>
+      </c>
+      <c r="D15" t="n">
+        <v>84611</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-19645</v>
+      </c>
+      <c r="F15" t="n">
+        <v>319</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-19326</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>45849</v>
+      </c>
+      <c r="B16" t="n">
+        <v>166243</v>
+      </c>
+      <c r="C16" t="n">
+        <v>73795</v>
+      </c>
+      <c r="D16" t="n">
+        <v>84692</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-19592</v>
+      </c>
+      <c r="F16" t="n">
+        <v>837</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-18755</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>45856</v>
+      </c>
+      <c r="B17" t="n">
+        <v>168569</v>
+      </c>
+      <c r="C17" t="n">
+        <v>75595</v>
+      </c>
+      <c r="D17" t="n">
+        <v>85266</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-19541</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1053</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-18488</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>45863</v>
+      </c>
+      <c r="B18" t="n">
+        <v>171848</v>
+      </c>
+      <c r="C18" t="n">
+        <v>78864</v>
+      </c>
+      <c r="D18" t="n">
+        <v>85223</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-19524</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1731</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-17793</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>45961</v>
+      </c>
+      <c r="B19" t="n">
+        <v>183598</v>
+      </c>
+      <c r="C19" t="n">
+        <v>72719</v>
+      </c>
+      <c r="D19" t="n">
+        <v>103215</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-19658</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2988</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-16670</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>45968</v>
+      </c>
+      <c r="B20" t="n">
+        <v>185047</v>
+      </c>
+      <c r="C20" t="n">
+        <v>74318</v>
+      </c>
+      <c r="D20" t="n">
+        <v>103061</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-17649</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2699</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-14950</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>45975</v>
+      </c>
+      <c r="B21" t="n">
+        <v>187432</v>
+      </c>
+      <c r="C21" t="n">
+        <v>72351</v>
+      </c>
+      <c r="D21" t="n">
+        <v>107389</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-17667</v>
+      </c>
+      <c r="F21" t="n">
+        <v>3275</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-14392</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>45982</v>
+      </c>
+      <c r="B22" t="n">
+        <v>180631</v>
+      </c>
+      <c r="C22" t="n">
+        <v>68580</v>
+      </c>
+      <c r="D22" t="n">
+        <v>104392</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-17620</v>
+      </c>
+      <c r="F22" t="n">
+        <v>3282</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-14338</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B23" t="n">
+        <v>147426</v>
+      </c>
+      <c r="C23" t="n">
+        <v>45537</v>
+      </c>
+      <c r="D23" t="n">
+        <v>94250</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-17667</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1806</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-15861</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B24" t="n">
+        <v>159694</v>
+      </c>
+      <c r="C24" t="n">
+        <v>54276</v>
+      </c>
+      <c r="D24" t="n">
+        <v>97742</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-17580</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2535</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-15045</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
         <v>46213</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B25" t="n">
         <v>163302</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C25" t="n">
         <v>59442</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D25" t="n">
         <v>96179</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E25" t="n">
         <v>-16577</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F25" t="n">
         <v>2836</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G25" t="n">
         <v>-13741</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Otomatik veri güncelleme (30.07.2026 13:16 UTC)
</commit_message>
<xml_diff>
--- a/net rezerv/likidite.xlsx
+++ b/net rezerv/likidite.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1032,6 +1032,29 @@
         <v>-13478</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B27" t="n">
+        <v>162606</v>
+      </c>
+      <c r="C27" t="n">
+        <v>54720</v>
+      </c>
+      <c r="D27" t="n">
+        <v>100210</v>
+      </c>
+      <c r="E27" t="n">
+        <v>-16555</v>
+      </c>
+      <c r="F27" t="n">
+        <v>3736</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-12819</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Otomatik veri güncelleme (20.08.2026 12:03 UTC)
</commit_message>
<xml_diff>
--- a/net rezerv/likidite.xlsx
+++ b/net rezerv/likidite.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1101,6 +1101,29 @@
         <v>-12421</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B30" t="n">
+        <v>183501</v>
+      </c>
+      <c r="C30" t="n">
+        <v>67445</v>
+      </c>
+      <c r="D30" t="n">
+        <v>108335</v>
+      </c>
+      <c r="E30" t="n">
+        <v>-16454</v>
+      </c>
+      <c r="F30" t="n">
+        <v>3595</v>
+      </c>
+      <c r="G30" t="n">
+        <v>-12859</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>